<commit_message>
sources: TAPP workbook sync, @id anyOf branches, guidance sidecars
- Workbooks synced from the authoritative Google Drive TAPPs: LA-Q v2->v3
  (renamed; +18 v3 rows), TEM/SEM_Imaging/SEM_FIBSEM content merges, and new
  Solution Q-ICP-MS / SF-ICP-MS v5 workbooks.
- tappDefinition + geochemProperties/instrument schema.yaml: add {@id} object
  branches to propertyID / additionalType anyOf (backward-compatible).
- docs/<workbook>.overrides.json: the minimal-annotation residual (curated
  names, analyte columns, technique-specific roles) for the 5 tier-column TAPPs.
- README / TAPP_TEMPLATE_GUIDE: v3 rename references.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SEM_Imaging_TAPP_v4.xlsx
+++ b/docs/SEM_Imaging_TAPP_v4.xlsx
@@ -2,24 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="351" yWindow="669" windowWidth="21849" windowHeight="9951" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TAPP" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legends" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'TAPP'!$C$1:$P$60</definedName>
-  </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,71 +27,36 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color rgb="FFC00000"/>
-      <sz val="11"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color rgb="FF0070C0"/>
-      <sz val="11"/>
+      <color rgb="000070C0"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color rgb="FF7030A0"/>
-      <sz val="11"/>
+      <color rgb="007030A0"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color rgb="FF375623"/>
-      <sz val="11"/>
+      <color rgb="00375623"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="11"/>
+      <color rgb="00000000"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color rgb="FFFF0000"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="10"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="7">
@@ -104,27 +68,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9D9D9"/>
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9E1F2"/>
+        <fgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -140,7 +104,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -202,21 +166,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -580,30 +532,60 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AZ60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12.53515625" customWidth="1" style="21" min="1" max="1"/>
-    <col width="25.23046875" customWidth="1" style="21" min="2" max="2"/>
-    <col width="10.3828125" customWidth="1" style="21" min="3" max="3"/>
-    <col width="11.07421875" customWidth="1" style="21" min="4" max="4"/>
-    <col width="9.765625" customWidth="1" style="21" min="5" max="5"/>
-    <col width="23.07421875" customWidth="1" style="21" min="6" max="6"/>
-    <col width="7.4609375" customWidth="1" style="21" min="7" max="7"/>
-    <col hidden="1" width="14" customWidth="1" style="21" min="8" max="8"/>
-    <col width="6.69140625" customWidth="1" style="21" min="9" max="9"/>
-    <col width="6.15234375" customWidth="1" style="21" min="10" max="10"/>
-    <col width="7.3046875" customWidth="1" style="21" min="11" max="11"/>
-    <col width="7.23046875" customWidth="1" style="21" min="12" max="12"/>
-    <col width="5.921875" customWidth="1" style="21" min="13" max="13"/>
-    <col width="27.23046875" customWidth="1" style="1" min="14" max="14"/>
-    <col width="23.921875" customWidth="1" style="21" min="15" max="15"/>
-    <col width="23.69140625" customWidth="1" style="21" min="16" max="16"/>
-    <col width="10.3828125" customWidth="1" style="21" min="17" max="17"/>
-    <col width="30" customWidth="1" style="21" min="18" max="49"/>
-    <col width="9.23046875" customWidth="1" style="21" min="50" max="16384"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="68" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="4" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="19" max="19"/>
+    <col width="30" customWidth="1" min="20" max="20"/>
+    <col width="30" customWidth="1" min="21" max="21"/>
+    <col width="30" customWidth="1" min="22" max="22"/>
+    <col width="30" customWidth="1" min="23" max="23"/>
+    <col width="30" customWidth="1" min="24" max="24"/>
+    <col width="30" customWidth="1" min="25" max="25"/>
+    <col width="30" customWidth="1" min="26" max="26"/>
+    <col width="30" customWidth="1" min="27" max="27"/>
+    <col width="30" customWidth="1" min="28" max="28"/>
+    <col width="30" customWidth="1" min="29" max="29"/>
+    <col width="30" customWidth="1" min="30" max="30"/>
+    <col width="30" customWidth="1" min="31" max="31"/>
+    <col width="30" customWidth="1" min="32" max="32"/>
+    <col width="30" customWidth="1" min="33" max="33"/>
+    <col width="30" customWidth="1" min="34" max="34"/>
+    <col width="30" customWidth="1" min="35" max="35"/>
+    <col width="30" customWidth="1" min="36" max="36"/>
+    <col width="30" customWidth="1" min="37" max="37"/>
+    <col width="30" customWidth="1" min="38" max="38"/>
+    <col width="30" customWidth="1" min="39" max="39"/>
+    <col width="30" customWidth="1" min="40" max="40"/>
+    <col width="30" customWidth="1" min="41" max="41"/>
+    <col width="30" customWidth="1" min="42" max="42"/>
+    <col width="30" customWidth="1" min="43" max="43"/>
+    <col width="30" customWidth="1" min="44" max="44"/>
+    <col width="30" customWidth="1" min="45" max="45"/>
+    <col width="30" customWidth="1" min="46" max="46"/>
+    <col width="30" customWidth="1" min="47" max="47"/>
+    <col width="30" customWidth="1" min="48" max="48"/>
+    <col width="30" customWidth="1" min="49" max="49"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40.85" customFormat="1" customHeight="1" s="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Metadata Item</t>
@@ -669,17 +651,17 @@
           <t>EBSD</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>schema path</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>matchComment</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>implementation notes</t>
         </is>
@@ -865,7 +847,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="29.15" customHeight="1">
+    <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
           <t>1. Protocol Identification</t>
@@ -903,46 +885,188 @@
           <t>N</t>
         </is>
       </c>
-      <c r="O2" s="1" t="n"/>
-      <c r="P2" s="1" t="n"/>
-      <c r="Q2" s="5" t="n"/>
-      <c r="R2" s="5" t="n"/>
-      <c r="S2" s="5" t="n"/>
-      <c r="T2" s="5" t="n"/>
-      <c r="U2" s="5" t="n"/>
-      <c r="V2" s="5" t="n"/>
-      <c r="W2" s="5" t="n"/>
-      <c r="X2" s="5" t="n"/>
-      <c r="Y2" s="5" t="n"/>
-      <c r="Z2" s="5" t="n"/>
-      <c r="AA2" s="5" t="n"/>
-      <c r="AB2" s="5" t="n"/>
-      <c r="AC2" s="5" t="n"/>
-      <c r="AD2" s="5" t="n"/>
-      <c r="AE2" s="5" t="n"/>
-      <c r="AF2" s="5" t="n"/>
-      <c r="AG2" s="5" t="n"/>
-      <c r="AH2" s="5" t="n"/>
-      <c r="AI2" s="5" t="n"/>
-      <c r="AJ2" s="5" t="n"/>
-      <c r="AK2" s="5" t="n"/>
-      <c r="AL2" s="5" t="n"/>
-      <c r="AM2" s="5" t="n"/>
-      <c r="AN2" s="5" t="n"/>
-      <c r="AO2" s="5" t="n"/>
-      <c r="AP2" s="5" t="n"/>
-      <c r="AQ2" s="5" t="n"/>
-      <c r="AR2" s="5" t="n"/>
-      <c r="AS2" s="5" t="n"/>
-      <c r="AT2" s="5" t="n"/>
-      <c r="AU2" s="5" t="n"/>
-      <c r="AV2" s="5" t="n"/>
-      <c r="AW2" s="5" t="n"/>
-      <c r="AX2" s="5" t="n"/>
-      <c r="AY2" s="5" t="n"/>
-      <c r="AZ2" s="5" t="n"/>
+      <c r="Q2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="T2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="V2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="W2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="X2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Y2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Z2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AC2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AD2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AE2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AF2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AG2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AH2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AI2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AJ2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AK2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AL2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AM2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AN2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AO2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AP2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AQ2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AR2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AS2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AT2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AU2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AV2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AX2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AZ2" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
-    <row r="3" ht="72.90000000000001" customHeight="1">
+    <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Protocol Name</t>
@@ -1004,17 +1128,16 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N3" s="1" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:name</t>
         </is>
       </c>
-      <c r="O3" s="1" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>methodDefinition.schema:name is the short descriptive name for the method.</t>
         </is>
       </c>
-      <c r="P3" s="1" t="n"/>
       <c r="Q3" s="9" t="inlineStr">
         <is>
           <t>N</t>
@@ -1196,7 +1319,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="72.90000000000001" customHeight="1">
+    <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Technique</t>
@@ -1258,17 +1381,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N4" s="1" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:measurementTechnique.schema:DefinedTerm.schema:termCode</t>
         </is>
       </c>
-      <c r="O4" s="1" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>methodDefinition.schema:measurementTechnique is a DefinedTerm; use .schema:termCode for the controlled-list code</t>
         </is>
       </c>
-      <c r="P4" s="1" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t xml:space="preserve">
 datatype: string
@@ -1456,7 +1579,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="58.3" customHeight="1">
+    <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Protocol Author</t>
@@ -1518,17 +1641,16 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N5" s="1" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:creator.schema:Person | schema.Organization.schema:name</t>
         </is>
       </c>
-      <c r="O5" s="1" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>schema:creator is a Person or Organization; schema:name carries the author name (plus schema:identifier for ORCID).</t>
         </is>
       </c>
-      <c r="P5" s="1" t="n"/>
       <c r="Q5" s="9" t="inlineStr">
         <is>
           <t>N</t>
@@ -1710,7 +1832,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="72.90000000000001" customHeight="1">
+    <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
           <t>Laboratory</t>
@@ -1772,17 +1894,16 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N6" s="1" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:location.scheme:Place.schema:name</t>
         </is>
       </c>
-      <c r="O6" s="1" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>ada:laboratory extends spatialExtent (schema:Place); schema:name is the lab/facility name.</t>
         </is>
       </c>
-      <c r="P6" s="1" t="n"/>
       <c r="Q6" s="9" t="inlineStr">
         <is>
           <t>N</t>
@@ -1964,7 +2085,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="43.75" customHeight="1">
+    <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
           <t>Laboratory ID</t>
@@ -2026,17 +2147,16 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N7" s="1" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:location.scheme:Place.schema:identifier</t>
         </is>
       </c>
-      <c r="O7" s="1" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>schema:Place schema:identifier (ROR or other PID) on ada:laboratory.</t>
         </is>
       </c>
-      <c r="P7" s="1" t="n"/>
       <c r="Q7" s="9" t="inlineStr">
         <is>
           <t>N</t>
@@ -2218,7 +2338,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="102" customHeight="1">
+    <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
           <t>Protocol Start Date</t>
@@ -2280,17 +2400,16 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N8" s="1" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:datePublished</t>
         </is>
       </c>
-      <c r="O8" s="1" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>match. methodDefinition.schema:datePublished is explicitly described as 'ISO 8601 date when this method configuration was first used'.</t>
         </is>
       </c>
-      <c r="P8" s="1" t="n"/>
       <c r="Q8" s="9" t="inlineStr">
         <is>
           <t>N</t>
@@ -2472,7 +2591,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="102" customHeight="1">
+    <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
           <t>Funding Source for Protocol Development</t>
@@ -2534,17 +2653,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N9" s="1" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:funding[].schema:MonetaryGrant.schema:name</t>
         </is>
       </c>
-      <c r="O9" s="1" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>match. schema:funding[] is an array of MonetaryGrant; also has schema:identifier (award number) and schema:funder (organisation).</t>
         </is>
       </c>
-      <c r="P9" s="1" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>put text in MonetaryGrant name unless can clearly parse identifier distinct from name.</t>
         </is>
@@ -2730,7 +2849,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="102" customHeight="1">
+    <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
           <t>Protocol Reference(s)</t>
@@ -2792,17 +2911,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N10" s="1" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:relatedLink[].schema:linkRelationship[name =  'techniquePublication'].</t>
         </is>
       </c>
-      <c r="O10" s="1" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>match. schema:relatedLink[] is a labeledLink with schema:url and schema:name; fits DOIs/URLs of method publications.</t>
         </is>
       </c>
-      <c r="P10" s="1" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>target URL to publication , target name should be title of publication</t>
         </is>
@@ -2988,7 +3107,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="72.90000000000001" customHeight="1">
+    <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
           <t>Protocol DOI</t>
@@ -3050,17 +3169,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N11" s="1" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>$Dataset.schema:measuremntTechnique.schema:DefinedTerm.schema.name and schema.identifier</t>
         </is>
       </c>
-      <c r="O11" s="1" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>This should be the identifier for the protocol definition that the analysis level 'detail' is extenting for a particular dataset.</t>
         </is>
       </c>
-      <c r="P11" s="1" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>required</t>
         </is>
@@ -3246,7 +3365,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="58.3" customHeight="1">
+    <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
           <t>Analyst</t>
@@ -3308,13 +3427,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N12" s="1" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>$Dataset.prov:wasGeneratedBy.schema:Agent/schema:Person.schema:name, schema:identifier</t>
         </is>
       </c>
-      <c r="O12" s="1" t="n"/>
-      <c r="P12" s="1" t="inlineStr">
+      <c r="P12" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -3500,7 +3618,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="29.15" customHeight="1">
+    <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
           <t>Analysis Start Date</t>
@@ -3562,13 +3680,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N13" s="1" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>$Dataset.prov:wasGeneratedBy.schema:startDate</t>
         </is>
       </c>
-      <c r="O13" s="1" t="n"/>
-      <c r="P13" s="1" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -3754,7 +3871,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="43.75" customHeight="1">
+    <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
           <t>Analysis End Date</t>
@@ -3816,13 +3933,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N14" s="1" t="inlineStr">
+      <c r="N14" t="inlineStr">
         <is>
           <t>$Dataset.prov:wasGeneratedBy.schema:endDate</t>
         </is>
       </c>
-      <c r="O14" s="1" t="n"/>
-      <c r="P14" s="1" t="inlineStr">
+      <c r="P14" t="inlineStr">
         <is>
           <t>optional</t>
         </is>
@@ -4008,7 +4124,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="43.75" customHeight="1">
+    <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
           <t>Funding Source for Analysis</t>
@@ -4070,13 +4186,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N15" s="1" t="inlineStr">
+      <c r="N15" t="inlineStr">
         <is>
           <t>$Dataset.schema:funding</t>
         </is>
       </c>
-      <c r="O15" s="1" t="n"/>
-      <c r="P15" s="1" t="inlineStr">
+      <c r="P15" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -4262,7 +4377,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="70.3" customHeight="1">
+    <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
           <t>Coupled Technique(s)</t>
@@ -4324,17 +4439,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N16" s="1" t="inlineStr">
+      <c r="N16" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:relatedLink[].schema:linkRelationship[name =  'coupledTechnique'].schema:target.schema:name</t>
         </is>
       </c>
-      <c r="O16" s="1" t="inlineStr">
+      <c r="O16" t="inlineStr">
         <is>
           <t>range should be analytical technique vocabulary</t>
         </is>
       </c>
-      <c r="P16" s="1" t="inlineStr">
+      <c r="P16" t="inlineStr">
         <is>
           <t>schema:DefinedTerm.schema:termCode
 datatype: string</t>
@@ -4521,7 +4636,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="102.9" customHeight="1">
+    <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
           <t>Coupling Description</t>
@@ -4583,13 +4698,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N17" s="1" t="inlineStr">
+      <c r="N17" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:relatedLink[].schema:linkRelationship[name =  'coupledTechnique'].schema:target.schema:description</t>
         </is>
       </c>
-      <c r="O17" s="1" t="n"/>
-      <c r="P17" s="1" t="inlineStr">
+      <c r="P17" t="inlineStr">
         <is>
           <t>text description of relationship</t>
         </is>
@@ -4775,7 +4889,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="72.90000000000001" customHeight="1">
+    <row r="18">
       <c r="A18" s="1" t="inlineStr">
         <is>
           <t>Coupled Protocol DOI</t>
@@ -4837,13 +4951,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N18" s="1" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>$Dataset.schema:relatedLink[].schema:linkRelationship[name =  'coupledTechnique'].schema:target.schema:url</t>
         </is>
       </c>
-      <c r="O18" s="1" t="n"/>
-      <c r="P18" s="1" t="n"/>
       <c r="Q18" s="9" t="inlineStr">
         <is>
           <t>N</t>
@@ -5025,7 +5137,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="102" customHeight="1">
+    <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
           <t>Coupled Dataset or Publication Reference</t>
@@ -5087,13 +5199,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N19" s="1" t="inlineStr">
+      <c r="N19" t="inlineStr">
         <is>
           <t>$Dataset.schema:relatedLink[].schema:linkRelationship[name =  'coupledDataset'].schema:target</t>
         </is>
       </c>
-      <c r="O19" s="1" t="n"/>
-      <c r="P19" s="1" t="n"/>
       <c r="Q19" s="9" t="inlineStr">
         <is>
           <t>N</t>
@@ -5313,46 +5423,188 @@
           <t>N</t>
         </is>
       </c>
-      <c r="O20" s="1" t="n"/>
-      <c r="P20" s="1" t="n"/>
-      <c r="Q20" s="5" t="n"/>
-      <c r="R20" s="5" t="n"/>
-      <c r="S20" s="5" t="n"/>
-      <c r="T20" s="5" t="n"/>
-      <c r="U20" s="5" t="n"/>
-      <c r="V20" s="5" t="n"/>
-      <c r="W20" s="5" t="n"/>
-      <c r="X20" s="5" t="n"/>
-      <c r="Y20" s="5" t="n"/>
-      <c r="Z20" s="5" t="n"/>
-      <c r="AA20" s="5" t="n"/>
-      <c r="AB20" s="5" t="n"/>
-      <c r="AC20" s="5" t="n"/>
-      <c r="AD20" s="5" t="n"/>
-      <c r="AE20" s="5" t="n"/>
-      <c r="AF20" s="5" t="n"/>
-      <c r="AG20" s="5" t="n"/>
-      <c r="AH20" s="5" t="n"/>
-      <c r="AI20" s="5" t="n"/>
-      <c r="AJ20" s="5" t="n"/>
-      <c r="AK20" s="5" t="n"/>
-      <c r="AL20" s="5" t="n"/>
-      <c r="AM20" s="5" t="n"/>
-      <c r="AN20" s="5" t="n"/>
-      <c r="AO20" s="5" t="n"/>
-      <c r="AP20" s="5" t="n"/>
-      <c r="AQ20" s="5" t="n"/>
-      <c r="AR20" s="5" t="n"/>
-      <c r="AS20" s="5" t="n"/>
-      <c r="AT20" s="5" t="n"/>
-      <c r="AU20" s="5" t="n"/>
-      <c r="AV20" s="5" t="n"/>
-      <c r="AW20" s="5" t="n"/>
-      <c r="AX20" s="5" t="n"/>
-      <c r="AY20" s="5" t="n"/>
-      <c r="AZ20" s="5" t="n"/>
+      <c r="Q20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="T20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="V20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="W20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="X20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Y20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Z20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AC20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AD20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AE20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AF20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AG20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AH20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AI20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AJ20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AK20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AL20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AM20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AN20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AO20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AP20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AQ20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AR20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AS20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AT20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AU20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AV20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AX20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AZ20" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
-    <row r="21" ht="145.75" customHeight="1">
+    <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
           <t>Target Material</t>
@@ -5414,17 +5666,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N21" s="1" t="inlineStr">
+      <c r="N21" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:object[].schema:DefinedTerm.schema.name</t>
         </is>
       </c>
-      <c r="O21" s="1" t="inlineStr">
+      <c r="O21" t="inlineStr">
         <is>
           <t>match. schema:object[] is an array of DefinedTerm or string describing target material (mineral phase, glass, oxide, etc.). Need vocabulary or target materials…</t>
         </is>
       </c>
-      <c r="P21" s="1" t="inlineStr">
+      <c r="P21" t="inlineStr">
         <is>
           <t>schema:DefinedTerm.schema:termCode
 datatype: enum {Silicate glass | Feldspar | Pyroxene | Olivine | Oxide | Sulfide | Carbonate | Phosphate | Native metal | Iron meteorite | Fluid inclusion | Melt inclusion | Whole rock | Other: specify}</t>
@@ -5611,7 +5863,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="134.6" customHeight="1">
+    <row r="22">
       <c r="A22" s="1" t="inlineStr">
         <is>
           <t>Sample Preparation Method</t>
@@ -5673,17 +5925,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N22" s="1" t="inlineStr">
+      <c r="N22" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:actionProcess.schema:step[][schema:name='samplePreparation'].schema:description</t>
         </is>
       </c>
-      <c r="O22" s="1" t="inlineStr">
+      <c r="O22" t="inlineStr">
         <is>
           <t>Sample preparation is a dedicated step (typically schema:position=1) in the actionProcess; schema:object is input, mostly likely the original sample. Schema:result is the product that will be used directly for analysis, e.g. polished thin section or epoxy mount; describe procedure in schema:step/schema:description</t>
         </is>
       </c>
-      <c r="P22" s="1" t="inlineStr">
+      <c r="P22" t="inlineStr">
         <is>
           <t>property:samplePreparationMethodDefault ;
 dataType: string ;
@@ -5871,7 +6123,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="102" customHeight="1">
+    <row r="23">
       <c r="A23" s="1" t="inlineStr">
         <is>
           <t>Sample Name</t>
@@ -5933,13 +6185,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N23" s="1" t="inlineStr">
+      <c r="N23" t="inlineStr">
         <is>
           <t>$Dataset.prov:wasGeneratedBy.schema:object[@type ="schema:Thing",            "https://w3id.org/isample/vocabulary/materialsampleobjecttype/materialsample"].schema:name</t>
         </is>
       </c>
-      <c r="O23" s="1" t="n"/>
-      <c r="P23" s="1" t="inlineStr">
+      <c r="P23" t="inlineStr">
         <is>
           <t>required</t>
         </is>
@@ -6125,7 +6376,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="102" customHeight="1">
+    <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
           <t>Sample Persistent Identifier</t>
@@ -6187,13 +6438,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N24" s="1" t="inlineStr">
+      <c r="N24" t="inlineStr">
         <is>
           <t>$Dataset.prov:wasGeneratedBy.schema:object[@type = "schema:Thing",  "https://w3id.org/isample/vocabulary/materialsampleobjecttype/materialsample"].schema:identifier</t>
         </is>
       </c>
-      <c r="O24" s="1" t="n"/>
-      <c r="P24" s="1" t="inlineStr">
+      <c r="P24" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
@@ -6379,7 +6629,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="29.15" customHeight="1">
+    <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
           <t>3. Instrument &amp; Software</t>
@@ -6417,46 +6667,188 @@
           <t>N</t>
         </is>
       </c>
-      <c r="O25" s="1" t="n"/>
-      <c r="P25" s="1" t="n"/>
-      <c r="Q25" s="5" t="n"/>
-      <c r="R25" s="5" t="n"/>
-      <c r="S25" s="5" t="n"/>
-      <c r="T25" s="5" t="n"/>
-      <c r="U25" s="5" t="n"/>
-      <c r="V25" s="5" t="n"/>
-      <c r="W25" s="5" t="n"/>
-      <c r="X25" s="5" t="n"/>
-      <c r="Y25" s="5" t="n"/>
-      <c r="Z25" s="5" t="n"/>
-      <c r="AA25" s="5" t="n"/>
-      <c r="AB25" s="5" t="n"/>
-      <c r="AC25" s="5" t="n"/>
-      <c r="AD25" s="5" t="n"/>
-      <c r="AE25" s="5" t="n"/>
-      <c r="AF25" s="5" t="n"/>
-      <c r="AG25" s="5" t="n"/>
-      <c r="AH25" s="5" t="n"/>
-      <c r="AI25" s="5" t="n"/>
-      <c r="AJ25" s="5" t="n"/>
-      <c r="AK25" s="5" t="n"/>
-      <c r="AL25" s="5" t="n"/>
-      <c r="AM25" s="5" t="n"/>
-      <c r="AN25" s="5" t="n"/>
-      <c r="AO25" s="5" t="n"/>
-      <c r="AP25" s="5" t="n"/>
-      <c r="AQ25" s="5" t="n"/>
-      <c r="AR25" s="5" t="n"/>
-      <c r="AS25" s="5" t="n"/>
-      <c r="AT25" s="5" t="n"/>
-      <c r="AU25" s="5" t="n"/>
-      <c r="AV25" s="5" t="n"/>
-      <c r="AW25" s="5" t="n"/>
-      <c r="AX25" s="5" t="n"/>
-      <c r="AY25" s="5" t="n"/>
-      <c r="AZ25" s="5" t="n"/>
+      <c r="Q25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="T25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="V25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="W25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="X25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Y25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Z25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AC25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AD25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AE25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AF25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AG25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AH25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AI25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AJ25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AK25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AL25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AM25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AN25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AO25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AP25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AQ25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AR25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AS25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AT25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AU25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AV25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AX25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AZ25" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
-    <row r="26" ht="102" customHeight="1">
+    <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
           <t>Instrument Manufacturer</t>
@@ -6518,17 +6910,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N26" s="1" t="inlineStr">
+      <c r="N26" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:instrument.schema:manufacturer.schema:Organization.schema:name</t>
         </is>
       </c>
-      <c r="O26" s="1" t="inlineStr">
+      <c r="O26" t="inlineStr">
         <is>
           <t>CDIF instrument inherits schema.org Product's schema:manufacturer.</t>
         </is>
       </c>
-      <c r="P26" s="1" t="inlineStr">
+      <c r="P26" t="inlineStr">
         <is>
           <t>DataType: string
 read-only: true
@@ -6716,7 +7108,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="87.45" customHeight="1">
+    <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
           <t>Instrument Model</t>
@@ -6778,17 +7170,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N27" s="1" t="inlineStr">
+      <c r="N27" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:instrument.schema:model.schema:name</t>
         </is>
       </c>
-      <c r="O27" s="1" t="inlineStr">
+      <c r="O27" t="inlineStr">
         <is>
           <t>CDIF instrument inherits schema.org Product's schema:model.</t>
         </is>
       </c>
-      <c r="P27" s="1" t="inlineStr">
+      <c r="P27" t="inlineStr">
         <is>
           <t>DataType: string
 read-only: true</t>
@@ -6975,7 +7367,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="145.75" customHeight="1">
+    <row r="28">
       <c r="A28" s="1" t="inlineStr">
         <is>
           <t>Electron Source</t>
@@ -7037,17 +7429,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N28" s="1" t="inlineStr">
+      <c r="N28" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:instrument.schema:hasPart[].additionalType = 'ElectronSource'</t>
         </is>
       </c>
-      <c r="O28" s="1" t="inlineStr">
+      <c r="O28" t="inlineStr">
         <is>
           <t>match. Electron source/gun modelled as a sub-component of the instrument via schema:hasPart[]; classify the part via schema:additionalType (e.g. 'ElectronGun:FEG') and carry the label in schema:name.</t>
         </is>
       </c>
-      <c r="P28" s="1" t="inlineStr">
+      <c r="P28" t="inlineStr">
         <is>
           <t>DataType: string
 read-only: true
@@ -7235,7 +7627,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="81" customHeight="1">
+    <row r="29">
       <c r="A29" s="1" t="inlineStr">
         <is>
           <t>Instrument Variant</t>
@@ -7297,13 +7689,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N29" s="1" t="inlineStr">
+      <c r="N29" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:instrument.schema:additionalType</t>
         </is>
       </c>
-      <c r="O29" s="1" t="n"/>
-      <c r="P29" s="1" t="inlineStr">
+      <c r="P29" t="inlineStr">
         <is>
           <t>DataType: string
 read-only: true
@@ -7491,7 +7882,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="80.59999999999999" customHeight="1">
+    <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
           <t>SE Detector Type</t>
@@ -7553,17 +7944,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="N30" s="1" t="inlineStr">
+      <c r="N30" t="inlineStr">
         <is>
           <t>$MethodDefinition.ada:seDetectorType</t>
         </is>
       </c>
-      <c r="O30" s="1" t="inlineStr">
+      <c r="O30" t="inlineStr">
         <is>
           <t>validation if exists ada:analysisMode = 'SE Imaging'</t>
         </is>
       </c>
-      <c r="P30" s="1" t="inlineStr">
+      <c r="P30" t="inlineStr">
         <is>
           <t>property: seDetectorType
 dataType: string ;
@@ -7752,7 +8143,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="119.15" customHeight="1">
+    <row r="31">
       <c r="A31" s="1" t="inlineStr">
         <is>
           <t>BSE Detector Type</t>
@@ -7814,17 +8205,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="N31" s="1" t="inlineStr">
+      <c r="N31" t="inlineStr">
         <is>
           <t>$MethodDefinition.ada:bseDetectorType</t>
         </is>
       </c>
-      <c r="O31" s="1" t="inlineStr">
+      <c r="O31" t="inlineStr">
         <is>
           <t>validation if exists ada:analysisMode = 'BSE Imaging'</t>
         </is>
       </c>
-      <c r="P31" s="1" t="inlineStr">
+      <c r="P31" t="inlineStr">
         <is>
           <t>property: bseDetectorType
 DataType: string
@@ -8013,7 +8404,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="145.75" customHeight="1">
+    <row r="32">
       <c r="A32" s="1" t="inlineStr">
         <is>
           <t>CL Detector Configuration</t>
@@ -8079,17 +8470,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="N32" s="1" t="inlineStr">
+      <c r="N32" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:additionalProperty[clDetectorConfiguration]</t>
         </is>
       </c>
-      <c r="O32" s="1" t="inlineStr">
+      <c r="O32" t="inlineStr">
         <is>
           <t xml:space="preserve">validation if exists [ada:analysisMode ='CL point analysis'] or [ada:analysisMode ='CL point analysis'] </t>
         </is>
       </c>
-      <c r="P32" s="1" t="inlineStr">
+      <c r="P32" t="inlineStr">
         <is>
           <t>parameter: clDetectorConfiguration
 dataType: string
@@ -8277,7 +8668,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="116.6" customHeight="1">
+    <row r="33">
       <c r="A33" s="1" t="inlineStr">
         <is>
           <t>EBSD Detector Configuration</t>
@@ -8343,17 +8734,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N33" s="1" t="inlineStr">
+      <c r="N33" t="inlineStr">
         <is>
           <t>$MethodDefinition.ada:ebsdDetectorConfiguration</t>
         </is>
       </c>
-      <c r="O33" s="1" t="inlineStr">
+      <c r="O33" t="inlineStr">
         <is>
           <t>validation if exists ada:analysisMode = 'EBSD'</t>
         </is>
       </c>
-      <c r="P33" s="1" t="inlineStr">
+      <c r="P33" t="inlineStr">
         <is>
           <t>property: ebsdDetectorConfiguration
 dataType: string
@@ -8541,7 +8932,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="131.15" customHeight="1">
+    <row r="34">
       <c r="A34" s="1" t="inlineStr">
         <is>
           <t>Acquisition Software</t>
@@ -8603,17 +8994,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N34" s="1" t="inlineStr">
+      <c r="N34" t="inlineStr">
         <is>
           <t>$MethodDefinition.bios:computationalTool[]</t>
         </is>
       </c>
-      <c r="O34" s="1" t="inlineStr">
+      <c r="O34" t="inlineStr">
         <is>
           <t>match. bios:computationalTool[] with ada:toolRole='acquisition' captures the acquisition/automation software; schema:name, schema:version, and schema:url are siblings.</t>
         </is>
       </c>
-      <c r="P34" s="1" t="inlineStr">
+      <c r="P34" t="inlineStr">
         <is>
           <t>toolRole = acquisition</t>
         </is>
@@ -8799,7 +9190,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="116.6" customHeight="1">
+    <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
           <t>Data Reduction Software</t>
@@ -8861,17 +9252,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N35" s="1" t="inlineStr">
+      <c r="N35" t="inlineStr">
         <is>
           <t>$MethodDefinition.bios:computationalTool[]</t>
         </is>
       </c>
-      <c r="O35" s="1" t="inlineStr">
+      <c r="O35" t="inlineStr">
         <is>
           <t>match. Same container as row 20 with ada:toolRole='reduction' for matrix-correction/data-reduction software.</t>
         </is>
       </c>
-      <c r="P35" s="1" t="inlineStr">
+      <c r="P35" t="inlineStr">
         <is>
           <t>toolRole = data reduction</t>
         </is>
@@ -9057,7 +9448,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="43.75" customHeight="1">
+    <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
           <t>4. Measurement Information</t>
@@ -9095,46 +9486,188 @@
           <t>N</t>
         </is>
       </c>
-      <c r="O36" s="1" t="n"/>
-      <c r="P36" s="1" t="n"/>
-      <c r="Q36" s="5" t="n"/>
-      <c r="R36" s="5" t="n"/>
-      <c r="S36" s="5" t="n"/>
-      <c r="T36" s="5" t="n"/>
-      <c r="U36" s="5" t="n"/>
-      <c r="V36" s="5" t="n"/>
-      <c r="W36" s="5" t="n"/>
-      <c r="X36" s="5" t="n"/>
-      <c r="Y36" s="5" t="n"/>
-      <c r="Z36" s="5" t="n"/>
-      <c r="AA36" s="5" t="n"/>
-      <c r="AB36" s="5" t="n"/>
-      <c r="AC36" s="5" t="n"/>
-      <c r="AD36" s="5" t="n"/>
-      <c r="AE36" s="5" t="n"/>
-      <c r="AF36" s="5" t="n"/>
-      <c r="AG36" s="5" t="n"/>
-      <c r="AH36" s="5" t="n"/>
-      <c r="AI36" s="5" t="n"/>
-      <c r="AJ36" s="5" t="n"/>
-      <c r="AK36" s="5" t="n"/>
-      <c r="AL36" s="5" t="n"/>
-      <c r="AM36" s="5" t="n"/>
-      <c r="AN36" s="5" t="n"/>
-      <c r="AO36" s="5" t="n"/>
-      <c r="AP36" s="5" t="n"/>
-      <c r="AQ36" s="5" t="n"/>
-      <c r="AR36" s="5" t="n"/>
-      <c r="AS36" s="5" t="n"/>
-      <c r="AT36" s="5" t="n"/>
-      <c r="AU36" s="5" t="n"/>
-      <c r="AV36" s="5" t="n"/>
-      <c r="AW36" s="5" t="n"/>
-      <c r="AX36" s="5" t="n"/>
-      <c r="AY36" s="5" t="n"/>
-      <c r="AZ36" s="5" t="n"/>
+      <c r="Q36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="T36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="V36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="W36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="X36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Y36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Z36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AC36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AD36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AE36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AF36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AG36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AH36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AI36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AJ36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AK36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AL36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AM36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AN36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AO36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AP36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AQ36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AR36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AS36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AT36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AU36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AV36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AX36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AZ36" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
-    <row r="37" ht="102" customHeight="1">
+    <row r="37">
       <c r="A37" s="1" t="inlineStr">
         <is>
           <t>Analytical Mode</t>
@@ -9196,17 +9729,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N37" s="1" t="inlineStr">
+      <c r="N37" t="inlineStr">
         <is>
           <t>$MethodDefinition.ada:analyticalMode</t>
         </is>
       </c>
-      <c r="O37" s="24" t="inlineStr">
+      <c r="O37" t="inlineStr">
         <is>
           <t>list in examples doesn't match options in columns I-M</t>
         </is>
       </c>
-      <c r="P37" s="1" t="inlineStr">
+      <c r="P37" t="inlineStr">
         <is>
           <t>property:analyticalMode
  dataType: string
@@ -9395,7 +9928,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="174.9" customHeight="1">
+    <row r="38">
       <c r="A38" s="1" t="inlineStr">
         <is>
           <t>Accelerating Voltage</t>
@@ -9457,17 +9990,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N38" s="1" t="inlineStr">
+      <c r="N38" t="inlineStr">
         <is>
           <t>$MethodDefinition.ada:acceleratingVoltage</t>
         </is>
       </c>
-      <c r="O38" s="1" t="inlineStr">
+      <c r="O38" t="inlineStr">
         <is>
           <t xml:space="preserve"> schema:unitText='kV'</t>
         </is>
       </c>
-      <c r="P38" s="1" t="inlineStr">
+      <c r="P38" t="inlineStr">
         <is>
           <t xml:space="preserve">property:  acceleratingVoltage
   datatype: string
@@ -9656,7 +10189,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="84.90000000000001" customHeight="1">
+    <row r="39">
       <c r="A39" s="1" t="inlineStr">
         <is>
           <t>Beam Current</t>
@@ -9722,13 +10255,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N39" s="23" t="inlineStr">
+      <c r="N39" t="inlineStr">
         <is>
           <t>$MethodDefinition.ada:beamCurrent</t>
         </is>
       </c>
-      <c r="O39" s="22" t="n"/>
-      <c r="P39" s="23" t="inlineStr">
+      <c r="P39" t="inlineStr">
         <is>
           <t>property: beamCurrent
  dataType: string
@@ -9916,7 +10448,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="47.15" customHeight="1">
+    <row r="40">
       <c r="A40" s="1" t="inlineStr">
         <is>
           <t>Working Distance</t>
@@ -9978,13 +10510,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N40" s="23" t="inlineStr">
+      <c r="N40" t="inlineStr">
         <is>
           <t>$MethodDefinition.ada:workingDistance</t>
         </is>
       </c>
-      <c r="O40" s="22" t="n"/>
-      <c r="P40" s="23" t="inlineStr">
+      <c r="P40" t="inlineStr">
         <is>
           <t>property: workingDistance
  dataType: string
@@ -10172,7 +10703,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="63" customHeight="1">
+    <row r="41">
       <c r="A41" s="1" t="inlineStr">
         <is>
           <t>Chamber Pressure</t>
@@ -10234,13 +10765,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N41" s="23" t="inlineStr">
+      <c r="N41" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:additionalProperty[chamberPressure].schema.name</t>
         </is>
       </c>
-      <c r="O41" s="22" t="n"/>
-      <c r="P41" s="23" t="inlineStr">
+      <c r="P41" t="inlineStr">
         <is>
           <t>parameter: chamberPressure
  dataType: string
@@ -10428,7 +10958,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="131.15" customHeight="1">
+    <row r="42">
       <c r="A42" s="1" t="inlineStr">
         <is>
           <t>Image Pixel Size</t>
@@ -10490,17 +11020,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="N42" s="23" t="inlineStr">
+      <c r="N42" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:additionalProperty[imagePixelSize].schema.name</t>
         </is>
       </c>
-      <c r="O42" s="1" t="inlineStr">
+      <c r="O42" t="inlineStr">
         <is>
           <t xml:space="preserve">validation if exists [ada:analysisMode ='SE Imaging'] or [ada:analysisMode ='BSE Imaging''] </t>
         </is>
       </c>
-      <c r="P42" s="23" t="inlineStr">
+      <c r="P42" t="inlineStr">
         <is>
           <t>parameter: imagePixelSize
  dataType: string
@@ -10688,7 +11218,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="62.6" customHeight="1">
+    <row r="43">
       <c r="A43" s="1" t="inlineStr">
         <is>
           <t>Dwell Time per Pixel</t>
@@ -10750,17 +11280,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="N43" s="23" t="inlineStr">
+      <c r="N43" t="inlineStr">
         <is>
           <t>$MethodDefinition.ada:dwellTimePerPixel</t>
         </is>
       </c>
-      <c r="O43" s="1" t="inlineStr">
+      <c r="O43" t="inlineStr">
         <is>
           <t xml:space="preserve">validation if exists [ada:analysisMode ='SE Imaging'] or [ada:analysisMode ='BSE Imaging''] </t>
         </is>
       </c>
-      <c r="P43" s="1" t="inlineStr">
+      <c r="P43" t="inlineStr">
         <is>
           <t>property: dwellTimePerPixel
  dataType: string
@@ -10948,7 +11478,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="160.3" customHeight="1">
+    <row r="44">
       <c r="A44" s="1" t="inlineStr">
         <is>
           <t>CL Acquisition Mode</t>
@@ -11014,17 +11544,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="N44" s="23" t="inlineStr">
+      <c r="N44" t="inlineStr">
         <is>
           <t>$MethodDefinition.ada:clAcquisitionMode</t>
         </is>
       </c>
-      <c r="O44" s="1" t="inlineStr">
+      <c r="O44" t="inlineStr">
         <is>
           <t xml:space="preserve">validation if exists [ada:analysisMode ='CL Point Analysis'] or [ada:analysisMode ='CL Mapping'] </t>
         </is>
       </c>
-      <c r="P44" s="1" t="inlineStr">
+      <c r="P44" t="inlineStr">
         <is>
           <t xml:space="preserve">property: clAcquisitionMode
  dataType: string
@@ -11214,7 +11744,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="72.90000000000001" customHeight="1">
+    <row r="45">
       <c r="A45" s="1" t="inlineStr">
         <is>
           <t>CL Wavelength Range</t>
@@ -11280,17 +11810,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="N45" s="23" t="inlineStr">
+      <c r="N45" t="inlineStr">
         <is>
           <t>$MethodDefinition.ada:clWavelengthRange</t>
         </is>
       </c>
-      <c r="O45" s="1" t="inlineStr">
+      <c r="O45" t="inlineStr">
         <is>
           <t xml:space="preserve">validation if exists [ada:analysisMode ='CL Point Analysis'] or [ada:analysisMode ='CL Mapping'] </t>
         </is>
       </c>
-      <c r="P45" s="1" t="inlineStr">
+      <c r="P45" t="inlineStr">
         <is>
           <t>property: clWavelengthRange
  dataType: string
@@ -11478,7 +12008,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="102" customHeight="1">
+    <row r="46">
       <c r="A46" s="1" t="inlineStr">
         <is>
           <t>CL Grating</t>
@@ -11544,17 +12074,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="N46" s="23" t="inlineStr">
+      <c r="N46" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:additionalProperty[clGrating].schema.name</t>
         </is>
       </c>
-      <c r="O46" s="1" t="inlineStr">
+      <c r="O46" t="inlineStr">
         <is>
           <t xml:space="preserve">validation if exists [ada:analysisMode ='CL Point Analysis'] or [ada:analysisMode ='CL Mapping'] </t>
         </is>
       </c>
-      <c r="P46" s="1" t="inlineStr">
+      <c r="P46" t="inlineStr">
         <is>
           <t>parameter: clWavelengthRange
  dataType: string
@@ -11742,7 +12272,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="116.6" customHeight="1">
+    <row r="47">
       <c r="A47" s="1" t="inlineStr">
         <is>
           <t>CL Integration Time</t>
@@ -11808,17 +12338,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="N47" s="23" t="inlineStr">
+      <c r="N47" t="inlineStr">
         <is>
           <t>$MethodDefinition.ada:clIntegrationTime</t>
         </is>
       </c>
-      <c r="O47" s="1" t="inlineStr">
+      <c r="O47" t="inlineStr">
         <is>
           <t xml:space="preserve">validation if exists [ada:analysisMode ='CL Point Analysis'] or [ada:analysisMode ='CL Mapping'] </t>
         </is>
       </c>
-      <c r="P47" s="1" t="inlineStr">
+      <c r="P47" t="inlineStr">
         <is>
           <t>property: clIntegrationTime
  dataType: string
@@ -12006,7 +12536,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="116.6" customHeight="1">
+    <row r="48">
       <c r="A48" s="1" t="inlineStr">
         <is>
           <t>Sample Tilt Angle</t>
@@ -12072,17 +12602,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N48" s="23" t="inlineStr">
+      <c r="N48" t="inlineStr">
         <is>
           <t>$MethodDefinition.ada:sampleTiltAngle</t>
         </is>
       </c>
-      <c r="O48" s="1" t="inlineStr">
+      <c r="O48" t="inlineStr">
         <is>
           <t>validation if exists [ada:analysisMode ='EBSD']</t>
         </is>
       </c>
-      <c r="P48" s="1" t="inlineStr">
+      <c r="P48" t="inlineStr">
         <is>
           <t>property: sampleTiltAngle
  dataType: string
@@ -12270,7 +12800,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="116.6" customHeight="1">
+    <row r="49">
       <c r="A49" s="1" t="inlineStr">
         <is>
           <t>EBSD Step Size</t>
@@ -12336,17 +12866,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N49" s="23" t="inlineStr">
+      <c r="N49" t="inlineStr">
         <is>
           <t>$MethodDefinition.ada:stepSize</t>
         </is>
       </c>
-      <c r="O49" s="1" t="inlineStr">
+      <c r="O49" t="inlineStr">
         <is>
           <t>validation if exists [ada:analysisMode ='EBSD']</t>
         </is>
       </c>
-      <c r="P49" s="1" t="inlineStr">
+      <c r="P49" t="inlineStr">
         <is>
           <t>property: stepSize
  dataType: string
@@ -12534,7 +13064,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="102" customHeight="1">
+    <row r="50">
       <c r="A50" s="1" t="inlineStr">
         <is>
           <t>EBSD Frame Time</t>
@@ -12600,17 +13130,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N50" s="23" t="inlineStr">
+      <c r="N50" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:additionalProperty[clFrameTime].schema.name</t>
         </is>
       </c>
-      <c r="O50" s="1" t="inlineStr">
+      <c r="O50" t="inlineStr">
         <is>
           <t>validation if exists [ada:analysisMode ='EBSD']</t>
         </is>
       </c>
-      <c r="P50" s="1" t="inlineStr">
+      <c r="P50" t="inlineStr">
         <is>
           <t>parameter: clFrameTime
  dataType: string
@@ -12798,7 +13328,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="116.6" customHeight="1">
+    <row r="51">
       <c r="A51" s="1" t="inlineStr">
         <is>
           <t>EBSD Phase List</t>
@@ -12864,17 +13394,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N51" s="23" t="inlineStr">
+      <c r="N51" t="inlineStr">
         <is>
           <t>$MethodDefinition.ada:phaseList[]</t>
         </is>
       </c>
-      <c r="O51" s="1" t="inlineStr">
+      <c r="O51" t="inlineStr">
         <is>
           <t>validation if exists [ada:analysisMode ='EBSD']</t>
         </is>
       </c>
-      <c r="P51" s="1" t="inlineStr">
+      <c r="P51" t="inlineStr">
         <is>
           <t>property: phaseList
  dataType: list of string
@@ -13062,7 +13592,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="29.15" customHeight="1">
+    <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
           <t>5. Data Processing</t>
@@ -13100,46 +13630,188 @@
           <t>N</t>
         </is>
       </c>
-      <c r="O52" s="1" t="n"/>
-      <c r="P52" s="1" t="n"/>
-      <c r="Q52" s="5" t="n"/>
-      <c r="R52" s="5" t="n"/>
-      <c r="S52" s="5" t="n"/>
-      <c r="T52" s="5" t="n"/>
-      <c r="U52" s="5" t="n"/>
-      <c r="V52" s="5" t="n"/>
-      <c r="W52" s="5" t="n"/>
-      <c r="X52" s="5" t="n"/>
-      <c r="Y52" s="5" t="n"/>
-      <c r="Z52" s="5" t="n"/>
-      <c r="AA52" s="5" t="n"/>
-      <c r="AB52" s="5" t="n"/>
-      <c r="AC52" s="5" t="n"/>
-      <c r="AD52" s="5" t="n"/>
-      <c r="AE52" s="5" t="n"/>
-      <c r="AF52" s="5" t="n"/>
-      <c r="AG52" s="5" t="n"/>
-      <c r="AH52" s="5" t="n"/>
-      <c r="AI52" s="5" t="n"/>
-      <c r="AJ52" s="5" t="n"/>
-      <c r="AK52" s="5" t="n"/>
-      <c r="AL52" s="5" t="n"/>
-      <c r="AM52" s="5" t="n"/>
-      <c r="AN52" s="5" t="n"/>
-      <c r="AO52" s="5" t="n"/>
-      <c r="AP52" s="5" t="n"/>
-      <c r="AQ52" s="5" t="n"/>
-      <c r="AR52" s="5" t="n"/>
-      <c r="AS52" s="5" t="n"/>
-      <c r="AT52" s="5" t="n"/>
-      <c r="AU52" s="5" t="n"/>
-      <c r="AV52" s="5" t="n"/>
-      <c r="AW52" s="5" t="n"/>
-      <c r="AX52" s="5" t="n"/>
-      <c r="AY52" s="5" t="n"/>
-      <c r="AZ52" s="5" t="n"/>
+      <c r="Q52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="T52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="V52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="W52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="X52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Y52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Z52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AC52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AD52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AE52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AF52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AG52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AH52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AI52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AJ52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AK52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AL52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AM52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AN52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AO52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AP52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AQ52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AR52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AS52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AT52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AU52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AV52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AX52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AZ52" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
-    <row r="53" ht="160.3" customHeight="1">
+    <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
           <t>EBSD Indexing Method</t>
@@ -13205,17 +13877,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N53" s="23" t="inlineStr">
+      <c r="N53" t="inlineStr">
         <is>
           <t>$MethodDefinition.ada:indexingMethod</t>
         </is>
       </c>
-      <c r="O53" s="1" t="inlineStr">
+      <c r="O53" t="inlineStr">
         <is>
           <t>validation if exists [ada:analysisMode ='EBSD']</t>
         </is>
       </c>
-      <c r="P53" s="1" t="inlineStr">
+      <c r="P53" t="inlineStr">
         <is>
           <t>property: indexingMethod
  dataType: string
@@ -13404,7 +14076,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="102" customHeight="1">
+    <row r="54">
       <c r="A54" s="1" t="inlineStr">
         <is>
           <t>Crystal Structure Database</t>
@@ -13470,17 +14142,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N54" s="23" t="inlineStr">
+      <c r="N54" t="inlineStr">
         <is>
           <t>$MethodDefinition.ada:crystalStructureDatabase</t>
         </is>
       </c>
-      <c r="O54" s="1" t="inlineStr">
+      <c r="O54" t="inlineStr">
         <is>
           <t>validation if exists [ada:analysisMode ='EBSD']</t>
         </is>
       </c>
-      <c r="P54" s="1" t="inlineStr">
+      <c r="P54" t="inlineStr">
         <is>
           <t>property: crystalStructureDatabase
  dataType: string
@@ -13668,7 +14340,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="116.6" customHeight="1">
+    <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
           <t>EBSD Pattern Quality Threshold</t>
@@ -13734,17 +14406,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N55" s="23" t="inlineStr">
+      <c r="N55" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:additionalProperty[patternQualityThreshold].schema.name</t>
         </is>
       </c>
-      <c r="O55" s="1" t="inlineStr">
+      <c r="O55" t="inlineStr">
         <is>
           <t>validation if exists [ada:analysisMode ='EBSD']</t>
         </is>
       </c>
-      <c r="P55" s="1" t="inlineStr">
+      <c r="P55" t="inlineStr">
         <is>
           <t>parameter: patternQualityThreshold
  dataType: string
@@ -13932,7 +14604,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="43.75" customHeight="1">
+    <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
           <t>6. Quality Control &amp; Uncertainty</t>
@@ -13970,46 +14642,188 @@
           <t>N</t>
         </is>
       </c>
-      <c r="O56" s="1" t="n"/>
-      <c r="P56" s="1" t="n"/>
-      <c r="Q56" s="5" t="n"/>
-      <c r="R56" s="5" t="n"/>
-      <c r="S56" s="5" t="n"/>
-      <c r="T56" s="5" t="n"/>
-      <c r="U56" s="5" t="n"/>
-      <c r="V56" s="5" t="n"/>
-      <c r="W56" s="5" t="n"/>
-      <c r="X56" s="5" t="n"/>
-      <c r="Y56" s="5" t="n"/>
-      <c r="Z56" s="5" t="n"/>
-      <c r="AA56" s="5" t="n"/>
-      <c r="AB56" s="5" t="n"/>
-      <c r="AC56" s="5" t="n"/>
-      <c r="AD56" s="5" t="n"/>
-      <c r="AE56" s="5" t="n"/>
-      <c r="AF56" s="5" t="n"/>
-      <c r="AG56" s="5" t="n"/>
-      <c r="AH56" s="5" t="n"/>
-      <c r="AI56" s="5" t="n"/>
-      <c r="AJ56" s="5" t="n"/>
-      <c r="AK56" s="5" t="n"/>
-      <c r="AL56" s="5" t="n"/>
-      <c r="AM56" s="5" t="n"/>
-      <c r="AN56" s="5" t="n"/>
-      <c r="AO56" s="5" t="n"/>
-      <c r="AP56" s="5" t="n"/>
-      <c r="AQ56" s="5" t="n"/>
-      <c r="AR56" s="5" t="n"/>
-      <c r="AS56" s="5" t="n"/>
-      <c r="AT56" s="5" t="n"/>
-      <c r="AU56" s="5" t="n"/>
-      <c r="AV56" s="5" t="n"/>
-      <c r="AW56" s="5" t="n"/>
-      <c r="AX56" s="5" t="n"/>
-      <c r="AY56" s="5" t="n"/>
-      <c r="AZ56" s="5" t="n"/>
+      <c r="Q56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="S56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="T56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="V56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="W56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="X56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Y56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Z56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AA56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AB56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AC56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AD56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AE56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AF56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AG56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AH56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AI56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AJ56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AK56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AL56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AM56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AN56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AO56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AP56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AQ56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AR56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AS56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AT56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AU56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AV56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AW56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AX56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AY56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="AZ56" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
-    <row r="57" ht="145.75" customHeight="1">
+    <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
           <t>EBSD Mean Angular Deviation</t>
@@ -14075,17 +14889,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N57" s="23" t="inlineStr">
+      <c r="N57" t="inlineStr">
         <is>
           <t>$Dataset.ada:meanAngularDeviaton</t>
         </is>
       </c>
-      <c r="O57" s="1" t="inlineStr">
+      <c r="O57" t="inlineStr">
         <is>
           <t>validation if exists [ada:analysisMode ='EBSD']</t>
         </is>
       </c>
-      <c r="P57" s="1" t="inlineStr">
+      <c r="P57" t="inlineStr">
         <is>
           <t>property: meanAngularDeviaton
  dataType: string
@@ -14273,7 +15087,7 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="131.15" customHeight="1">
+    <row r="58">
       <c r="A58" s="1" t="inlineStr">
         <is>
           <t>EBSD Indexing Rate</t>
@@ -14339,17 +15153,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N58" s="23" t="inlineStr">
+      <c r="N58" t="inlineStr">
         <is>
           <t>$Dataset.ada:indexingRate</t>
         </is>
       </c>
-      <c r="O58" s="1" t="inlineStr">
+      <c r="O58" t="inlineStr">
         <is>
           <t>validation if exists [ada:analysisMode ='EBSD']</t>
         </is>
       </c>
-      <c r="P58" s="1" t="inlineStr">
+      <c r="P58" t="inlineStr">
         <is>
           <t>property: indexingRate
  dataType: string
@@ -14537,7 +15351,7 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="102" customHeight="1">
+    <row r="59">
       <c r="A59" s="1" t="inlineStr">
         <is>
           <t>CL Wavelength Calibration Reference</t>
@@ -14603,17 +15417,17 @@
           <t>N</t>
         </is>
       </c>
-      <c r="N59" s="23" t="inlineStr">
+      <c r="N59" t="inlineStr">
         <is>
           <t>$MethodDefinition.schema:additionalProperty[clWavelengthCalibrationReference].schema.name</t>
         </is>
       </c>
-      <c r="O59" s="1" t="inlineStr">
+      <c r="O59" t="inlineStr">
         <is>
           <t xml:space="preserve">validation if exists [ada:analysisMode ='CL Point Analysis'] or [ada:analysisMode ='CL Mapping'] </t>
         </is>
       </c>
-      <c r="P59" s="1" t="inlineStr">
+      <c r="P59" t="inlineStr">
         <is>
           <t>parameter: clWavelengthCalibrationReference
  dataType: string
@@ -14801,7 +15615,7 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="110.25" customHeight="1">
+    <row r="60">
       <c r="A60" s="1" t="inlineStr">
         <is>
           <t>Additional Notes</t>
@@ -14863,17 +15677,17 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="N60" s="1" t="inlineStr">
+      <c r="N60" t="inlineStr">
         <is>
           <t>$.schema:description</t>
         </is>
       </c>
-      <c r="O60" s="1" t="inlineStr">
+      <c r="O60" t="inlineStr">
         <is>
           <t>method Property: schema:description accepts free-text narrative; additional notes can extend it or be distributed to the most relevant workflow step's schema:description.</t>
         </is>
       </c>
-      <c r="P60" s="1" t="inlineStr">
+      <c r="P60" t="inlineStr">
         <is>
           <t>method property : description
   datatype: text
@@ -15062,57 +15876,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="C1:P60"/>
-  <conditionalFormatting sqref="N53:N54">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFFFFFF"/>
-        <color rgb="FF57BB8A"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N55">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFFFFFF"/>
-        <color rgb="FF57BB8A"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N57:N58">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFFFFFF"/>
-        <color rgb="FF57BB8A"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N59">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFFFFFF"/>
-        <color rgb="FF57BB8A"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N39:P41 P42 N42:N51">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFFFFFF"/>
-        <color rgb="FF57BB8A"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15124,7 +15887,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
@@ -15132,7 +15895,7 @@
     <col width="55" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.9" customHeight="1">
+    <row r="1">
       <c r="A1" s="14" t="inlineStr">
         <is>
           <t>Protocol-Level Tier</t>
@@ -15154,7 +15917,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="72.90000000000001" customHeight="1">
+    <row r="2">
       <c r="A2" s="15" t="inlineStr">
         <is>
           <t>Basic</t>
@@ -15176,7 +15939,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="72.90000000000001" customHeight="1">
+    <row r="3">
       <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Advanced</t>
@@ -15198,7 +15961,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="43.75" customHeight="1">
+    <row r="4">
       <c r="A4" s="19" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -15220,7 +15983,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="29.15" customHeight="1">
+    <row r="5">
       <c r="C5" s="17" t="inlineStr">
         <is>
           <t>Advanced</t>
@@ -15232,7 +15995,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15.9" customHeight="1">
+    <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
           <t>Mode Column</t>

</xml_diff>